<commit_message>
feat(F-NAR-019): ATOM-DIF.ENE.001-06 La file du cerceau
Réécriture vocale example4 : éclat de lacet, énergie vécue.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.ENE.001-06.xlsx
+++ b/stories/arbres/ATOM-DIF.ENE.001-06.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le bateau-feuille</t>
+          <t>La file du cerceau</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin de l'école, bac sous l'arbre</t>
+          <t>cour d'école puis jardin, ombre d'arbre, cloche lointaine, cerceau rouge dans l'herbe, lacet, gourde, file</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut faire flotter une feuille jaune dans le bac. Chouchou arrive avec beaucoup d'énergie. L'eau éclabousse. Ils jouent, ils attendent, Amir demande à papa. La feuille tourne, tout lentement.</t>
+          <t>Le lacet glisse. Papa noue. Sur le nœud, un éclat de lacet brille. Cloche lointaine, ombre, cerceau rouge dans l'herbe. Amir veut la file, maintenant. Chouchou saute trop. Le cerceau part. Sourire parti. Il refuse de foncer. Merci vécu. Racine, elle veut passer. Il s'arrête, lit l'éclat. Un éclat de lacet tient sur le nœud.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une craie blanche a roulé sous le banc. Elle a un ventre cassé. Un morceau reste, tout sec. L'ombre du grand arbre fait des taches par terre. Une cloche lointaine fait ding, tout loin. Papa noue un lacet. Ton lacet est prêt, Amir ? Oui, papa. Maman glisse une gourde dans le sac. L'eau est fraîche. En ce moment, Amir ramasse une feuille jaune. Elle est sèche. Elle a des nervures. Elle craque un tout petit peu. Je veux un bateau. Dans le bac. Le bac est sous l'arbre. Amir souffle sur la feuille. Elle tremble dans sa main. Les chaussures tapent le sol de la cour. Chouchou arrive en sautant. Elle a beaucoup d'énergie. Elle tourne. Elle s'arrête. Elle recommence. Elle saute tout le temps. C'est son énergie. Ce n'est pas une faute. Ils font une file pour le bac. Chouchou a envie d'aller vite. L'eau éclabousse un peu. Ma feuille. La feuille jaune tremble au bord. Amir regarde papa.</t>
+          <t>Le lacet glisse entre les doigts de papa. Le bout plastique fait clic, sec et petit. Ça a fait clic ! Ton lacet, Amir ? Oui, papa. Papa noue le nœud, un peu serré. Sur le nœud, un éclat de lacet brille. Il brille, papa. Tu le vois, sur le nœud ? Oui, un petit point. La cour sent l'herbe chaude, un peu. Ça sent l'herbe, maman. Tes chaussures tiennent, Amir ? Oui, maman. Une cloche lointaine fait ding, loin dans l'air. J'ai entendu le ding. La cloche, Amir ? Oui, loin. L'ombre de l'arbre est longue, sur la cour. Maman glisse une gourde dans le sac. L'eau est fraîche. Elle est froide, maman. Ils passent de la cour au jardin. L'herbe est haute, un peu sèche. Je veux le cerceau, maintenant ! Le cerceau dans l'herbe ? Oui, tout de suite. Jusqu'à l'arbre ? Oui, maman. Un cerceau rouge repose dans l'herbe. Le plastique est tiède, un peu rêche. Il est chaud, papa. Tu le tiens, Amir ? Oui, papa. En ce moment, Amir tient le cerceau. Ils font une file vers l'arbre. Moi d'abord, maintenant ! Les chaussures tapent le sol, depuis la cour. Chouchou arrive en sautant. J'arrive ! Chouchou ! Elle saute sur place, trop vite. Le cerceau ! Moi, le cerceau, maintenant ! Chouchou prend le cerceau rouge. Elle le fait tourner trop vite. Le cerceau part vers la gourde. Il part ! Oh. Le cerceau tombe dans l'herbe. Ça fait un bruit mou. Il est tombé ! L'éclat de lacet tremble, puis tient. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Chouchou, Amir ? Oui, papa. Tes mains sont chaudes, Amir ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une craie blanche a roulé sous le banc. Elle a un ventre cassé. Un morceau reste, tout sec. L'ombre du grand arbre fait des taches par terre. Une cloche lointaine fait ding, tout loin. Papa noue un lacet. Ton lacet est prêt, Amir ? Oui, papa. Maman glisse une gourde dans le sac. L'eau est fraîche. En ce moment, Amir ramasse une feuille jaune. Elle est sèche. Elle a des nervures. Elle craque un tout petit peu. Je veux un bateau. Dans le bac. Le bac est sous l'arbre. Amir souffle sur la feuille. Elle tremble dans sa main. Les chaussures tapent le sol de la cour. Chouchou arrive en sautant. Elle a beaucoup d'énergie. Elle tourne. Elle s'arrête. Elle recommence. Elle saute tout le temps. C'est son énergie. Ce n'est pas une faute. Ils font une file pour le bac. Chouchou a envie d'aller vite. L'eau éclabousse un peu. Ma feuille. La feuille jaune tremble au bord. Amir regarde papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le lacet glisse entre les doigts de papa. Le bout plastique fait clic, sec et petit. Ça a fait clic ! Ton lacet, Amir ? Oui, papa. Papa noue le nœud, un peu serré. Sur le nœud, un &lt;emphasis level="moderate"&gt;éclat de lacet&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur le nœud ? Oui, un petit point. La cour sent l'herbe chaude, un peu. Ça sent l'herbe, maman. Tes chaussures tiennent, Amir ? Oui, maman. Une cloche lointaine fait ding, loin dans l'air. J'ai entendu le ding. La cloche, Amir ? Oui, loin. L'ombre de l'arbre est longue, sur la cour. Maman glisse une gourde dans le sac. L'eau est fraîche. Elle est froide, maman. Ils passent de la cour au jardin. L'herbe est haute, un peu sèche. Je veux le cerceau, maintenant ! Le cerceau dans l'herbe ? Oui, tout de suite. Jusqu'à l'arbre ? Oui, maman. Un cerceau rouge repose dans l'herbe. Le plastique est tiède, un peu rêche. Il est chaud, papa. Tu le tiens, Amir ? Oui, papa. En ce moment, Amir tient le cerceau. Ils font une file vers l'arbre. Moi d'abord, maintenant ! Les chaussures tapent le sol, depuis la cour. Chouchou arrive en sautant. J'arrive ! Chouchou ! Elle saute sur place, trop vite. Le cerceau ! Moi, le cerceau, maintenant ! Chouchou prend le cerceau rouge. Elle le fait tourner trop vite. Le cerceau part vers la gourde. Il part ! Oh. Le cerceau tombe dans l'herbe. Ça fait un bruit mou. Il est tombé ! L'éclat de lacet tremble, puis tient. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Chouchou, Amir ? Oui, papa. Tes mains sont chaudes, Amir ? Un peu, maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Maman laisse Baptiste dans la cour. Les chaussures tapent le sol. Noa arrive en sautant. Il a beaucoup d'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Il tourne. Il s'arrête. Il recommence. Baptiste le regarde. Maman est encore près du portail. Elle dit : beaucoup d'énergie, ce n'est pas une faute. On peut jouer. On peut attendre. On peut demander à un adulte. Baptiste hoche la tête. Ils font une file pour le cerceau. Noa a envie d'aller vite. Baptiste dit : on peut attendre. Noa souffle. Il reste dans la file. Ils jouent. Plus tard, au jardin de l'école, Noa a encore de l'énergie. Ce n'est pas une faute. Baptiste va vers la maîtresse. Il demande à un adulte. La maîtresse marche avec Noa jusqu'au bac. L'eau est froide. Puis ils versent l'eau ensemble. On peut jouer ou attendre. Maman revient. Baptiste dit : Noa a de l'énergie. Maman dit : ce n'est pas une faute. [pause]</t>
+          <t>Le lacet glisse entre les doigts de papa. Le bout plastique fait clic, sec et petit. Ça a fait clic ! Ton lacet, Amir ? Oui, papa. Papa noue le nœud, un peu serré. Sur le nœud, un &lt;emphasis&gt;éclat de lacet&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur le nœud ? Oui, un petit point. La cour sent l'herbe chaude, un peu. Ça sent l'herbe, maman. Tes chaussures tiennent, Amir ? Oui, maman. Une cloche lointaine fait ding, loin dans l'air. J'ai entendu le ding. La cloche, Amir ? Oui, loin. L'ombre de l'arbre est longue, sur la cour. Maman glisse une gourde dans le sac. L'eau est fraîche. Elle est froide, maman. Ils passent de la cour au jardin. L'herbe est haute, un peu sèche. Je veux le cerceau, maintenant ! Le cerceau dans l'herbe ? Oui, tout de suite. Jusqu'à l'arbre ? Oui, maman. Un cerceau rouge repose dans l'herbe. Le plastique est tiède, un peu rêche. Il est chaud, papa. Tu le tiens, Amir ? Oui, papa. En ce moment, Amir tient le cerceau. Ils font une file vers l'arbre. Moi d'abord, maintenant ! Les chaussures tapent le sol, depuis la cour. Chouchou arrive en sautant. J'arrive ! Chouchou ! Elle saute sur place, trop vite. Le cerceau ! Moi, le cerceau, maintenant ! Chouchou prend le cerceau rouge. Elle le fait tourner trop vite. Le cerceau part vers la gourde. Il part ! Oh. Le cerceau tombe dans l'herbe. Ça fait un bruit mou. Il est tombé ! L'éclat de lacet tremble, puis tient. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Chouchou, Amir ? Oui, papa. Tes mains sont chaudes, Amir ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>éclat de lacet</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,43 +1321,74 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_file_du_cerceau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une craie blanche a roulé sous le banc.
-narrateur|Elle a un ventre cassé.
-narrateur|Un morceau reste, tout sec.
-narrateur|L'ombre du grand arbre fait des taches par terre.
-narrateur|Une cloche lointaine fait ding, tout loin.
-narrateur|Papa noue un lacet.
-papa|Ton lacet est prêt, Amir ?
+          <t>narrateur|Le lacet glisse entre les doigts de papa.
+narrateur|Le bout plastique fait clic, sec et petit.
+enfant-m|Ça a fait clic !
+papa|Ton lacet, Amir ?
 enfant-m|Oui, papa.
+narrateur|Papa noue le nœud, un peu serré.
+narrateur|Sur le nœud, un éclat de lacet brille.
+enfant-m|Il brille, papa.
+papa|Tu le vois, sur le nœud ?
+enfant-m|Oui, un petit point.
+narrateur|La cour sent l'herbe chaude, un peu.
+enfant-m|Ça sent l'herbe, maman.
+maman|Tes chaussures tiennent, Amir ?
+enfant-m|Oui, maman.
+narrateur|Une cloche lointaine fait ding, loin dans l'air.
+enfant-m|J'ai entendu le ding.
+papa|La cloche, Amir ?
+enfant-m|Oui, loin.
+narrateur|L'ombre de l'arbre est longue, sur la cour.
 narrateur|Maman glisse une gourde dans le sac.
 maman|L'eau est fraîche.
-narrateur|En ce moment, Amir ramasse une feuille jaune.
-narrateur|Elle est sèche.
-narrateur|Elle a des nervures.
-narrateur|Elle craque un tout petit peu.
-enfant-m|Je veux un bateau.
-enfant-m|Dans le bac.
-papa|Le bac est sous l'arbre.
-narrateur|Amir souffle sur la feuille.
-narrateur|Elle tremble dans sa main.
-narrateur|Les chaussures tapent le sol de la cour.
+enfant-m|Elle est froide, maman.
+narrateur|Ils passent de la cour au jardin.
+narrateur|L'herbe est haute, un peu sèche.
+enfant-m|Je veux le cerceau, maintenant !
+papa|Le cerceau dans l'herbe ?
+enfant-m|Oui, tout de suite.
+maman|Jusqu'à l'arbre ?
+enfant-m|Oui, maman.
+narrateur|Un cerceau rouge repose dans l'herbe.
+narrateur|Le plastique est tiède, un peu rêche.
+enfant-m|Il est chaud, papa.
+papa|Tu le tiens, Amir ?
+enfant-m|Oui, papa.
+narrateur|En ce moment, Amir tient le cerceau.
+narrateur|Ils font une file vers l'arbre.
+enfant-m|Moi d'abord, maintenant !
+narrateur|Les chaussures tapent le sol, depuis la cour.
 narrateur|Chouchou arrive en sautant.
-narrateur|Elle a beaucoup d'énergie.
-narrateur|Elle tourne.
-narrateur|Elle s'arrête.
-narrateur|Elle recommence.
-enfant-m|Elle saute tout le temps.
-maman|C'est son énergie.
-maman|Ce n'est pas une faute.
-narrateur|Ils font une file pour le bac.
-narrateur|Chouchou a envie d'aller vite.
-narrateur|L'eau éclabousse un peu.
-enfant-m|Ma feuille.
-narrateur|La feuille jaune tremble au bord.
-narrateur|Amir regarde papa.</t>
+copine|J'arrive !
+enfant-m|Chouchou !
+narrateur|Elle saute sur place, trop vite.
+copine|Le cerceau !
+enfant-m|Moi, le cerceau, maintenant !
+narrateur|Chouchou prend le cerceau rouge.
+narrateur|Elle le fait tourner trop vite.
+narrateur|Le cerceau part vers la gourde.
+enfant-m|Il part !
+copine|Oh.
+narrateur|Le cerceau tombe dans l'herbe.
+narrateur|Ça fait un bruit mou.
+enfant-m|Il est tombé !
+narrateur|L'éclat de lacet tremble, puis tient.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Chouchou, Amir ?
+enfant-m|Oui, papa.
+maman|Tes mains sont chaudes, Amir ?
+enfant-m|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1394,12 +1425,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a de l'énergie. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Chouchou a de l'&lt;emphasis level="moderate"&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Noa a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Chouchou a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1462,18 +1493,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1488,11 +1519,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1503,23 +1534,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1528,23 +1559,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=chouchou_a_de_l_energie_que_peut_on_faire; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1577,17 +1608,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir va vers papa. Papa, on fait quoi ? On fait flotter le bateau. On attend dans la file. Tu es venu me demander. On marche jusqu'au bac. Papa marche avec Chouchou. L'eau est froide. Chouchou pose les mains un moment. Elle souffle. L'énergie est encore là. Ce n'est pas une faute. On peut attendre. Chouchou reste dans la file. Amir pose la feuille sur l'eau. Elle tourne, tout lentement. On la laisse flotter ? Oui. Chouchou regarde la feuille. Elle attend. Puis elle pousse une toute petite vague. La feuille avance. Ils jouent. Amir attend son tour pour verser. Il verse un filet. La feuille fait un tour. Chacun son tour. Encore un tour. Encore un, tout doux. Une petite araignée d'eau part. La feuille la suit, tout lentement. Elle avance. Votre bateau a un sillage.</t>
+          <t>Amir veut le cerceau, tout de suite. Je le prends, maintenant ! Il avance trop vite vers Chouchou. Les mots se bousculent dans sa bouche. Attends. Chouchou saute, trop près de l'herbe. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il referme les mains. Personne ne parle. Il observe le cerceau, un instant. Il écoute la cloche, loin dans l'air. Tu veux le cerceau avec Chouchou ? Papa reste à la même hauteur. Papa, on fait quoi ? On reste dans la file ? Oui. On marche jusqu'à l'arbre ? Oui, maman. Viens, Chouchou. J'y vais. Ils restent dans la file, un moment. L'herbe froisse, sous les chaussures. L'herbe, papa. Tu poses les mains ? Oui. Amir pose les mains sur le plastique. Le cerceau est tiède. Chouchou pose les mains aussi. Il est chaud. Elle souffle. Merci, Amir. Papa a vu les deux, dans l'herbe. L'ombre de l'arbre a bougé, un peu. Elle est longue. Chouchou pose le cerceau, sans se presser. À toi. D'accord. Amir fait rouler le cerceau. Le cerceau passe dans l'herbe. Il roule ! Oui. Tu le vois, le rond rouge ? Oui, papa. Tes chaussures tiennent ? Oui, maman. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près de l'arbre ? Oui. Tes mains sont chaudes ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir va vers papa. Papa, on fait quoi ? On fait flotter le bateau. On attend dans la file. Tu es venu me demander. On marche jusqu'au bac. Papa marche avec Chouchou. L'eau est froide. Chouchou pose les mains un moment. Elle souffle. L'énergie est encore là. Ce n'est pas une faute. On peut attendre. Chouchou reste dans la file. Amir pose la feuille sur l'eau. Elle tourne, tout lentement. On la laisse flotter ? Oui. Chouchou regarde la feuille. Elle attend. Puis elle pousse une toute petite vague. La feuille avance. Ils jouent. Amir attend son tour pour verser. Il verse un filet. La feuille fait un tour. Chacun son tour. Encore un tour. Encore un, tout doux. Une petite araignée d'eau part. La feuille la suit, tout lentement. Elle avance. Votre bateau a un sillage.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir veut le &lt;emphasis level="moderate"&gt;cerceau&lt;/emphasis&gt;, tout de suite. Je le prends, maintenant ! Il avance trop vite vers Chouchou. Les mots se bousculent dans sa bouche. Attends. Chouchou saute, trop près de l'herbe. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il referme les mains. Personne ne parle. Il observe le cerceau, un instant. Il écoute la cloche, loin dans l'air. Tu veux le cerceau avec Chouchou ? Papa reste à la même hauteur. Papa, on fait quoi ? On reste dans la file ? Oui. On marche jusqu'à l'arbre ? Oui, maman. Viens, Chouchou. J'y vais. Ils restent dans la file, un moment. L'herbe froisse, sous les chaussures. L'herbe, papa. Tu poses les mains ? Oui. Amir pose les mains sur le plastique. Le cerceau est tiède. Chouchou pose les mains aussi. Il est chaud. Elle souffle. Merci, Amir. Papa a vu les deux, dans l'herbe. L'ombre de l'arbre a bougé, un peu. Elle est longue. Chouchou pose le cerceau, sans se presser. À toi. D'accord. Amir fait rouler le cerceau. Le cerceau passe dans l'herbe. Il roule ! Oui. Tu le vois, le rond rouge ? Oui, papa. Tes chaussures tiennent ? Oui, maman. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près de l'arbre ? Oui. Tes mains sont chaudes ? Un peu, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Noa a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Ce n'est pas une faute. Baptiste a joué. Il a su attendre. Il a demandé à un adulte. [pause]</t>
+          <t>Amir veut le &lt;emphasis&gt;cerceau&lt;/emphasis&gt;, tout de suite. Je le prends, maintenant ! Il avance trop vite vers Chouchou. Les mots se bousculent dans sa bouche. Attends. Chouchou saute, trop près de l'herbe. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il referme les mains. Personne ne parle. Il observe le cerceau, un instant. Il écoute la cloche, loin dans l'air. Tu veux le cerceau avec Chouchou ? Papa reste à la même hauteur. Papa, on fait quoi ? On reste dans la file ? Oui. On marche jusqu'à l'arbre ? Oui, maman. Viens, Chouchou. J'y vais. Ils restent dans la file, un moment. L'herbe froisse, sous les chaussures. L'herbe, papa. Tu poses les mains ? Oui. Amir pose les mains sur le plastique. Le cerceau est tiède. Chouchou pose les mains aussi. Il est chaud. Elle souffle. Merci, Amir. Papa a vu les deux, dans l'herbe. L'ombre de l'arbre a bougé, un peu. Elle est longue. Chouchou pose le cerceau, sans se presser. À toi. D'accord. Amir fait rouler le cerceau. Le cerceau passe dans l'herbe. Il roule ! Oui. Tu le vois, le rond rouge ? Oui, papa. Tes chaussures tiennent ? Oui, maman. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près de l'arbre ? Oui. Tes mains sont chaudes ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1634,7 +1665,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1642,10 +1673,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1668,30 +1699,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>cerceau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1700,10 +1731,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1716,44 +1747,64 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_reste_dans_la_file_avec_elle; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir va vers papa.
+          <t>narrateur|Amir veut le cerceau, tout de suite.
+enfant-m|Je le prends, maintenant !
+narrateur|Il avance trop vite vers Chouchou.
+narrateur|Les mots se bousculent dans sa bouche.
+copine|Attends.
+narrateur|Chouchou saute, trop près de l'herbe.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Amir refuse de foncer.
+narrateur|Il referme les mains.
+narrateur|Personne ne parle.
+narrateur|Il observe le cerceau, un instant.
+narrateur|Il écoute la cloche, loin dans l'air.
+papa|Tu veux le cerceau avec Chouchou ?
+narrateur|Papa reste à la même hauteur.
 enfant-m|Papa, on fait quoi ?
-papa|On fait flotter le bateau.
-papa|On attend dans la file.
-papa|Tu es venu me demander.
-papa|On marche jusqu'au bac.
-narrateur|Papa marche avec Chouchou.
-narrateur|L'eau est froide.
-narrateur|Chouchou pose les mains un moment.
+papa|On reste dans la file ?
+enfant-m|Oui.
+maman|On marche jusqu'à l'arbre ?
+enfant-m|Oui, maman.
+papa|Viens, Chouchou.
+copine|J'y vais.
+narrateur|Ils restent dans la file, un moment.
+narrateur|L'herbe froisse, sous les chaussures.
+enfant-m|L'herbe, papa.
+papa|Tu poses les mains ?
+enfant-m|Oui.
+narrateur|Amir pose les mains sur le plastique.
+narrateur|Le cerceau est tiède.
+narrateur|Chouchou pose les mains aussi.
+copine|Il est chaud.
 narrateur|Elle souffle.
-maman|L'énergie est encore là.
-maman|Ce n'est pas une faute.
-enfant-m|On peut attendre.
-narrateur|Chouchou reste dans la file.
-narrateur|Amir pose la feuille sur l'eau.
-narrateur|Elle tourne, tout lentement.
-papa|On la laisse flotter ?
+papa|Merci, Amir.
+narrateur|Papa a vu les deux, dans l'herbe.
+maman|L'ombre de l'arbre a bougé, un peu.
+enfant-m|Elle est longue.
+narrateur|Chouchou pose le cerceau, sans se presser.
+copine|À toi.
+enfant-m|D'accord.
+narrateur|Amir fait rouler le cerceau.
+narrateur|Le cerceau passe dans l'herbe.
+enfant-m|Il roule !
+copine|Oui.
+papa|Tu le vois, le rond rouge ?
+enfant-m|Oui, papa.
+maman|Tes chaussures tiennent ?
+enfant-m|Oui, maman.
+narrateur|Le ventre d'Amir se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près de l'arbre ?
 enfant-m|Oui.
-narrateur|Chouchou regarde la feuille.
-narrateur|Elle attend.
-narrateur|Puis elle pousse une toute petite vague.
-narrateur|La feuille avance.
-narrateur|Ils jouent.
-narrateur|Amir attend son tour pour verser.
-narrateur|Il verse un filet.
-narrateur|La feuille fait un tour.
-maman|Chacun son tour.
-enfant-f|Encore un tour.
-papa|Encore un, tout doux.
-narrateur|Une petite araignée d'eau part.
-narrateur|La feuille la suit, tout lentement.
-enfant-m|Elle avance.
-maman|Votre bateau a un sillage.</t>
+maman|Tes mains sont chaudes ?
+enfant-m|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1785,17 +1836,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On reprend le sac ? Oui, maman. Maman prend la main d'Amir. Chouchou ramasse le morceau de craie. Vous vous dites au revoir ? Au revoir. Au revoir, Chouchou. La feuille reste un moment sur l'eau. Ton bateau a voyagé. Tout autour du bac. On la laisse là ? Elle sèche sur le bord.</t>
+          <t>Ils vont sous l'arbre, dans le jardin. Une file, maintenant ! L'ombre glisse sur l'herbe. Chouchou veut passer, trop vite. Elle saute vers le tronc. Moi d'abord ! Le cerceau penche vers une racine. Ça tombe ! Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le cerceau, un instant. Il écoute la cloche, loin dans l'air. Sur le nœud, un éclat de lacet luit. Là, sur le nœud. Tu restes, Chouchou ? Chouchou ne dit rien. Elle souffle, sans parler. Oui. Elle reste derrière lui. Le cerceau, maman ? Le rouge, Amir. Amir pousse, sans se presser. Le cerceau contourne la racine. À moi. Chouchou pousse à son tour. Tu as soufflé, Chouchou ? Un peu. L'ombre est fraîche, Amir ? Un peu, maman. Vous roulez ensemble ? Oui, papa. Ils roulent le cerceau jusqu'au tronc. Le plastique tape le bois, sans bruit. Il est arrivé. Il est arrivé. Le cerceau a de l'herbe, Amir ? Sur le bord.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On reprend le sac ? Oui, maman. Maman prend la main d'Amir. Chouchou ramasse le morceau de craie. Vous vous dites au revoir ? Au revoir. Au revoir, Chouchou. La feuille reste un moment sur l'eau. Ton bateau a voyagé. Tout autour du bac. On la laisse là ? Elle sèche sur le bord.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils vont sous l'arbre, dans le jardin. Une file, maintenant ! L'ombre glisse sur l'herbe. Chouchou veut passer, trop vite. Elle saute vers le tronc. Moi d'abord ! Le cerceau penche vers une racine. Ça tombe ! Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le cerceau, un instant. Il écoute la cloche, loin dans l'air. Sur le nœud, un &lt;emphasis level="moderate"&gt;éclat de lacet&lt;/emphasis&gt; luit. Là, sur le nœud. Tu restes, Chouchou ? Chouchou ne dit rien. Elle souffle, sans parler. Oui. Elle reste derrière lui. Le cerceau, maman ? Le rouge, Amir. Amir pousse, sans se presser. Le cerceau contourne la racine. À moi. Chouchou pousse à son tour. Tu as soufflé, Chouchou ? Un peu. L'ombre est fraîche, Amir ? Un peu, maman. Vous roulez ensemble ? Oui, papa. Ils roulent le cerceau jusqu'au tronc. Le plastique tape le bois, sans bruit. Il est arrivé. Il est arrivé. Le cerceau a de l'herbe, Amir ? Sur le bord.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman prend la &lt;emphasis&gt;main&lt;/emphasis&gt; de Baptiste. Noa range un cerceau. [pause]</t>
+          <t>Ils vont sous l'arbre, dans le jardin. Une file, maintenant ! L'ombre glisse sur l'herbe. Chouchou veut passer, trop vite. Elle saute vers le tronc. Moi d'abord ! Le cerceau penche vers une racine. Ça tombe ! Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le cerceau, un instant. Il écoute la cloche, loin dans l'air. Sur le nœud, un &lt;emphasis&gt;éclat de lacet&lt;/emphasis&gt; luit. Là, sur le nœud. Tu restes, Chouchou ? Chouchou ne dit rien. Elle souffle, sans parler. Oui. Elle reste derrière lui. Le cerceau, maman ? Le rouge, Amir. Amir pousse, sans se presser. Le cerceau contourne la racine. À moi. Chouchou pousse à son tour. Tu as soufflé, Chouchou ? Un peu. L'ombre est fraîche, Amir ? Un peu, maman. Vous roulez ensemble ? Oui, papa. Ils roulent le cerceau jusqu'au tronc. Le plastique tape le bois, sans bruit. Il est arrivé. Il est arrivé. Le cerceau a de l'herbe, Amir ? Sur le bord. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1842,7 +1893,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1850,10 +1901,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1876,30 +1927,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de lacet</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1908,10 +1959,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1922,21 +1973,58 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_racine_elle_souffle; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On reprend le sac ?
-enfant-m|Oui, maman.
-narrateur|Maman prend la main d'Amir.
-narrateur|Chouchou ramasse le morceau de craie.
-papa|Vous vous dites au revoir ?
-enfant-f|Au revoir.
-enfant-m|Au revoir, Chouchou.
-narrateur|La feuille reste un moment sur l'eau.
-papa|Ton bateau a voyagé.
-enfant-m|Tout autour du bac.
-maman|On la laisse là ?
-enfant-m|Elle sèche sur le bord.</t>
+          <t>narrateur|Ils vont sous l'arbre, dans le jardin.
+enfant-m|Une file, maintenant !
+narrateur|L'ombre glisse sur l'herbe.
+narrateur|Chouchou veut passer, trop vite.
+narrateur|Elle saute vers le tronc.
+copine|Moi d'abord !
+narrateur|Le cerceau penche vers une racine.
+enfant-m|Ça tombe !
+narrateur|Amir avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Amir refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le cerceau, un instant.
+narrateur|Il écoute la cloche, loin dans l'air.
+narrateur|Sur le nœud, un éclat de lacet luit.
+enfant-m|Là, sur le nœud.
+enfant-m|Tu restes, Chouchou ?
+narrateur|Chouchou ne dit rien.
+narrateur|Elle souffle, sans parler.
+copine|Oui.
+narrateur|Elle reste derrière lui.
+enfant-m|Le cerceau, maman ?
+maman|Le rouge, Amir.
+narrateur|Amir pousse, sans se presser.
+narrateur|Le cerceau contourne la racine.
+copine|À moi.
+narrateur|Chouchou pousse à son tour.
+papa|Tu as soufflé, Chouchou ?
+copine|Un peu.
+maman|L'ombre est fraîche, Amir ?
+enfant-m|Un peu, maman.
+papa|Vous roulez ensemble ?
+enfant-m|Oui, papa.
+narrateur|Ils roulent le cerceau jusqu'au tronc.
+narrateur|Le plastique tape le bois, sans bruit.
+enfant-m|Il est arrivé.
+copine|Il est arrivé.
+maman|Le cerceau a de l'herbe, Amir ?
+enfant-m|Sur le bord.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1963,17 +2051,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La feuille jaune sèche sur le bord. L'ombre de l'arbre a bougé. Le bateau a fini son tour. Il a flotté.</t>
+          <t>Ils restent près de l'arbre. Maman essuie un peu d'herbe. On a eu le cerceau, papa. Tu l'as vu, toi ? Oui, jusqu'au tronc. On est bien, ici. Amir tapote le plastique du doigt. Il a une trace d'herbe. Tu la vois, la trace ? Oui, maman. Le cerceau est resté, Amir. Oui, avec Chouchou. Le cerceau est resté. Ça sent l'herbe, un peu tiède. Et le lacet, maman. Oui, dans l'air. Les chaussures restent dans l'herbe. Un éclat de lacet tient sur le nœud.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La feuille jaune sèche sur le bord. L'ombre de l'arbre a bougé. Le bateau a fini son tour. Il a flotté.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de l'arbre. Maman essuie un peu d'herbe. On a eu le cerceau, papa. Tu l'as vu, toi ? Oui, jusqu'au tronc. On est bien, ici. Amir tapote le plastique du doigt. Il a une trace d'herbe. Tu la vois, la trace ? Oui, maman. Le cerceau est resté, Amir. Oui, avec Chouchou. Le cerceau est resté. Ça sent l'herbe, un peu tiède. Et le lacet, maman. Oui, dans l'air. Les chaussures restent dans l'herbe. Un &lt;emphasis level="moderate"&gt;éclat de lacet&lt;/emphasis&gt; tient sur le nœud.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de l'arbre. Maman essuie un peu d'herbe. On a eu le cerceau, papa. Tu l'as vu, toi ? Oui, jusqu'au tronc. On est bien, ici. Amir tapote le plastique du doigt. Il a une trace d'herbe. Tu la vois, la trace ? Oui, maman. Le cerceau est resté, Amir. Oui, avec Chouchou. Le cerceau est resté. Ça sent l'herbe, un peu tiède. Et le lacet, maman. Oui, dans l'air. Les chaussures restent dans l'herbe. Un &lt;emphasis&gt;éclat de lacet&lt;/emphasis&gt; tient sur le nœud.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2020,18 +2108,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2040,12 +2128,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2054,17 +2142,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de lacet</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2073,11 +2165,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2086,27 +2178,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_noeud; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La feuille jaune sèche sur le bord.
-narrateur|L'ombre de l'arbre a bougé.
-papa|Le bateau a fini son tour.
-enfant-m|Il a flotté.</t>
+          <t>narrateur|Ils restent près de l'arbre.
+narrateur|Maman essuie un peu d'herbe.
+enfant-m|On a eu le cerceau, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, jusqu'au tronc.
+maman|On est bien, ici.
+narrateur|Amir tapote le plastique du doigt.
+enfant-m|Il a une trace d'herbe.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|Le cerceau est resté, Amir.
+enfant-m|Oui, avec Chouchou.
+copine|Le cerceau est resté.
+narrateur|Ça sent l'herbe, un peu tiède.
+enfant-m|Et le lacet, maman.
+maman|Oui, dans l'air.
+narrateur|Les chaussures restent dans l'herbe.
+narrateur|Un éclat de lacet tient sur le nœud.</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2212,6 +2322,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>